<commit_message>
Updated ETH_grids_kan10 model - 2026-06-18 22:54
</commit_message>
<xml_diff>
--- a/VerveStacks_ETH_grids_kan10/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_ETH_grids_kan10/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_ETH_grids_kan10\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{EFEC49AA-C2B4-485E-BAE7-FA3B5772C56A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{89F7F0CD-0F4E-48E7-85F7-03DF5D1BC832}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -19957,7 +19957,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8BBBC059-8F81-4BB0-88A8-610C8F08C7C0}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8E0F7A80-C102-488A-A698-6CC5EBA8FA09}">
   <dimension ref="B9:H91"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -21615,7 +21615,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{12E44ABF-9445-45F4-8579-E6B9569C3AEF}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D81E6303-B1F4-4C35-8282-0ACA58106F1F}">
   <dimension ref="B9:L91"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>